<commit_message>
Update test queries: replace placeholder names (ABC Traders, XYZ Distributors) with real customer name Valencia Tex (altaf Bhai)
</commit_message>
<xml_diff>
--- a/langsmith-tool-evaluator/Copilot Test Cases ---Surana Polycot.xlsx
+++ b/langsmith-tool-evaluator/Copilot Test Cases ---Surana Polycot.xlsx
@@ -886,14 +886,14 @@
     <row r="27" ht="30.75" customHeight="1">
       <c r="A27" s="12" t="inlineStr">
         <is>
-          <t>Show me the ledger of ABC Traders and summarize their account status.</t>
+          <t>Show me the ledger of Valencia Tex (altaf Bhai) and summarize their account status.</t>
         </is>
       </c>
     </row>
     <row r="28" ht="30.75" customHeight="1">
       <c r="A28" s="12" t="inlineStr">
         <is>
-          <t>Retrieve the ledger for Dhana Traders and explain the outstanding entries.</t>
+          <t>Retrieve the ledger for Valencia Tex (altaf Bhai) and explain the outstanding entries.</t>
         </is>
       </c>
     </row>
@@ -914,7 +914,7 @@
     <row r="31">
       <c r="A31" s="12" t="inlineStr">
         <is>
-          <t>Compare the ledgers of ABC Traders and XYZ Distributors.</t>
+          <t>Compare the ledgers of Valencia Tex (altaf Bhai) and Valencia Tex (altaf Bhai).</t>
         </is>
       </c>
     </row>

</xml_diff>